<commit_message>
feat: connect parser evaluation to final golden template
</commit_message>
<xml_diff>
--- a/outputs/golden_annotation_final/Golden_Annotation_Final.xlsx
+++ b/outputs/golden_annotation_final/Golden_Annotation_Final.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_Me" sheetId="1" r:id="Rff849178526d4c1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workbook_Info" sheetId="2" r:id="R21f9e1835d654d47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet_Annotation" sheetId="3" r:id="R146252114ff945e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_Annotation" sheetId="4" r:id="R42e860856c0d463c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Header_Annotation" sheetId="5" r:id="Rc875fa8317774f04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cell_Truth" sheetId="6" r:id="R4c2f31c3f8d54903"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Significance_Parsing_Cases" sheetId="7" r:id="R5913488c95184716"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_Me" sheetId="1" r:id="R2eb905db17b74f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workbook_Info" sheetId="2" r:id="Rbaf372ce76854665"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet_Annotation" sheetId="3" r:id="Rc71344d428cc40cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_Annotation" sheetId="4" r:id="R253e369303e34583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Header_Annotation" sheetId="5" r:id="R90e0582164b747e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cell_Truth" sheetId="6" r:id="R7d37dffff06f4522"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Significance_Parsing_Cases" sheetId="7" r:id="R140100a1467b4b17"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29864,6 +29864,2922 @@
         <x:v>AB621</x:v>
       </x:c>
     </x:row>
+    <x:row r="809">
+      <x:c r="A809" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B809" s="4" t="str">
+        <x:v>Q04_01_H2</x:v>
+      </x:c>
+      <x:c r="C809" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D809" s="4" t="str">
+        <x:v>Total</x:v>
+      </x:c>
+      <x:c r="E809" s="4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F809" s="4" t="str"/>
+      <x:c r="G809" s="4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H809" s="4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="I809" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J809" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K809" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L809" s="4" t="str">
+        <x:v>B10,B11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="810">
+      <x:c r="A810" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B810" s="4" t="str">
+        <x:v>Q04_01_H3</x:v>
+      </x:c>
+      <x:c r="C810" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D810" s="4" t="str">
+        <x:v>1~2线·有孩家庭</x:v>
+      </x:c>
+      <x:c r="E810" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F810" s="4" t="str"/>
+      <x:c r="G810" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H810" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="I810" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J810" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K810" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L810" s="4" t="str">
+        <x:v>C10,C11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="811">
+      <x:c r="A811" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B811" s="4" t="str">
+        <x:v>Q04_01_H4</x:v>
+      </x:c>
+      <x:c r="C811" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="D811" s="4" t="str">
+        <x:v>1~2线·其他家庭</x:v>
+      </x:c>
+      <x:c r="E811" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F811" s="4" t="str"/>
+      <x:c r="G811" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H811" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I811" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="J811" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="K811" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L811" s="4" t="str">
+        <x:v>D10,D11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="812">
+      <x:c r="A812" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B812" s="4" t="str">
+        <x:v>Q04_01_H5</x:v>
+      </x:c>
+      <x:c r="C812" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="D812" s="4" t="str">
+        <x:v>3线及以下</x:v>
+      </x:c>
+      <x:c r="E812" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="F812" s="4" t="str"/>
+      <x:c r="G812" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="H812" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="I812" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="J812" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="K812" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L812" s="4" t="str">
+        <x:v>E10,E11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="813">
+      <x:c r="A813" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B813" s="4" t="str">
+        <x:v>Q04_01_H6</x:v>
+      </x:c>
+      <x:c r="C813" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D813" s="4" t="str">
+        <x:v>低温用户</x:v>
+      </x:c>
+      <x:c r="E813" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="F813" s="4" t="str"/>
+      <x:c r="G813" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="H813" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="I813" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="J813" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="K813" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L813" s="4" t="str">
+        <x:v>F10,F11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="814">
+      <x:c r="A814" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B814" s="4" t="str">
+        <x:v>Q04_01_H7</x:v>
+      </x:c>
+      <x:c r="C814" s="4" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="D814" s="4" t="str">
+        <x:v>仅常温用户</x:v>
+      </x:c>
+      <x:c r="E814" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F814" s="4" t="str"/>
+      <x:c r="G814" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H814" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I814" s="4" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="J814" s="4" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="K814" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L814" s="4" t="str">
+        <x:v>G10,G11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="815">
+      <x:c r="A815" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B815" s="4" t="str">
+        <x:v>Q04_01_H8</x:v>
+      </x:c>
+      <x:c r="C815" s="4" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="D815" s="4" t="str">
+        <x:v>低温 Total</x:v>
+      </x:c>
+      <x:c r="E815" s="4" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="F815" s="4" t="str"/>
+      <x:c r="G815" s="4" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="H815" s="4" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="I815" s="4" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="J815" s="4" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="K815" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L815" s="4" t="str">
+        <x:v>H10,H11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="816">
+      <x:c r="A816" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B816" s="4" t="str">
+        <x:v>Q04_01_H9</x:v>
+      </x:c>
+      <x:c r="C816" s="4" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D816" s="4" t="str">
+        <x:v>1~2线·有孩家庭</x:v>
+      </x:c>
+      <x:c r="E816" s="4" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="F816" s="4" t="str"/>
+      <x:c r="G816" s="4" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="H816" s="4" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="I816" s="4" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="J816" s="4" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="K816" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L816" s="4" t="str">
+        <x:v>I10,I11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="817">
+      <x:c r="A817" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B817" s="4" t="str">
+        <x:v>Q04_01_H10</x:v>
+      </x:c>
+      <x:c r="C817" s="4" t="str">
+        <x:v>J</x:v>
+      </x:c>
+      <x:c r="D817" s="4" t="str">
+        <x:v>1~2线·其他家庭</x:v>
+      </x:c>
+      <x:c r="E817" s="4" t="str">
+        <x:v>c</x:v>
+      </x:c>
+      <x:c r="F817" s="4" t="str"/>
+      <x:c r="G817" s="4" t="str">
+        <x:v>c</x:v>
+      </x:c>
+      <x:c r="H817" s="4" t="str">
+        <x:v>c</x:v>
+      </x:c>
+      <x:c r="I817" s="4" t="str">
+        <x:v>J</x:v>
+      </x:c>
+      <x:c r="J817" s="4" t="str">
+        <x:v>J</x:v>
+      </x:c>
+      <x:c r="K817" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L817" s="4" t="str">
+        <x:v>J10,J11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="818">
+      <x:c r="A818" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B818" s="4" t="str">
+        <x:v>Q04_01_H11</x:v>
+      </x:c>
+      <x:c r="C818" s="4" t="str">
+        <x:v>K</x:v>
+      </x:c>
+      <x:c r="D818" s="4" t="str">
+        <x:v>3线及以下</x:v>
+      </x:c>
+      <x:c r="E818" s="4" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="F818" s="4" t="str"/>
+      <x:c r="G818" s="4" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="H818" s="4" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="I818" s="4" t="str">
+        <x:v>K</x:v>
+      </x:c>
+      <x:c r="J818" s="4" t="str">
+        <x:v>K</x:v>
+      </x:c>
+      <x:c r="K818" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L818" s="4" t="str">
+        <x:v>K10,K11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="819">
+      <x:c r="A819" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B819" s="4" t="str">
+        <x:v>Q04_01_H12</x:v>
+      </x:c>
+      <x:c r="C819" s="4" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D819" s="4" t="str">
+        <x:v>L1 忠诚</x:v>
+      </x:c>
+      <x:c r="E819" s="4" t="str">
+        <x:v>e</x:v>
+      </x:c>
+      <x:c r="F819" s="4" t="str"/>
+      <x:c r="G819" s="4" t="str">
+        <x:v>e</x:v>
+      </x:c>
+      <x:c r="H819" s="4" t="str">
+        <x:v>e</x:v>
+      </x:c>
+      <x:c r="I819" s="4" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="J819" s="4" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="K819" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L819" s="4" t="str">
+        <x:v>L10,L11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="820">
+      <x:c r="A820" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B820" s="4" t="str">
+        <x:v>Q04_01_H13</x:v>
+      </x:c>
+      <x:c r="C820" s="4" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D820" s="4" t="str">
+        <x:v>L2 复购</x:v>
+      </x:c>
+      <x:c r="E820" s="4" t="str">
+        <x:v>f</x:v>
+      </x:c>
+      <x:c r="F820" s="4" t="str"/>
+      <x:c r="G820" s="4" t="str">
+        <x:v>f</x:v>
+      </x:c>
+      <x:c r="H820" s="4" t="str">
+        <x:v>f</x:v>
+      </x:c>
+      <x:c r="I820" s="4" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="J820" s="4" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="K820" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L820" s="4" t="str">
+        <x:v>M10,M11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="821">
+      <x:c r="A821" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B821" s="4" t="str">
+        <x:v>Q04_01_H14</x:v>
+      </x:c>
+      <x:c r="C821" s="4" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="D821" s="4" t="str">
+        <x:v>L3 试用</x:v>
+      </x:c>
+      <x:c r="E821" s="4" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="F821" s="4" t="str"/>
+      <x:c r="G821" s="4" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="H821" s="4" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="I821" s="4" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="J821" s="4" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="K821" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L821" s="4" t="str">
+        <x:v>N10,N11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="822">
+      <x:c r="A822" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B822" s="4" t="str">
+        <x:v>Q04_01_H15</x:v>
+      </x:c>
+      <x:c r="C822" s="4" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="D822" s="4" t="str">
+        <x:v>L4 错配</x:v>
+      </x:c>
+      <x:c r="E822" s="4" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="F822" s="4" t="str"/>
+      <x:c r="G822" s="4" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="H822" s="4" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="I822" s="4" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="J822" s="4" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="K822" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L822" s="4" t="str">
+        <x:v>O10,O11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="823">
+      <x:c r="A823" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B823" s="4" t="str">
+        <x:v>Q04_01_H16</x:v>
+      </x:c>
+      <x:c r="C823" s="4" t="str">
+        <x:v>P</x:v>
+      </x:c>
+      <x:c r="D823" s="4" t="str">
+        <x:v>L5 未买益生菌</x:v>
+      </x:c>
+      <x:c r="E823" s="4" t="str">
+        <x:v>i</x:v>
+      </x:c>
+      <x:c r="F823" s="4" t="str"/>
+      <x:c r="G823" s="4" t="str">
+        <x:v>i</x:v>
+      </x:c>
+      <x:c r="H823" s="4" t="str">
+        <x:v>i</x:v>
+      </x:c>
+      <x:c r="I823" s="4" t="str">
+        <x:v>P</x:v>
+      </x:c>
+      <x:c r="J823" s="4" t="str">
+        <x:v>P</x:v>
+      </x:c>
+      <x:c r="K823" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L823" s="4" t="str">
+        <x:v>P10,P11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="824">
+      <x:c r="A824" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B824" s="4" t="str">
+        <x:v>Q04_01_H17</x:v>
+      </x:c>
+      <x:c r="C824" s="4" t="str">
+        <x:v>Q</x:v>
+      </x:c>
+      <x:c r="D824" s="4" t="str">
+        <x:v>伊利 畅轻利乐冠系列</x:v>
+      </x:c>
+      <x:c r="E824" s="4" t="str">
+        <x:v>j</x:v>
+      </x:c>
+      <x:c r="F824" s="4" t="str"/>
+      <x:c r="G824" s="4" t="str">
+        <x:v>j</x:v>
+      </x:c>
+      <x:c r="H824" s="4" t="str">
+        <x:v>j</x:v>
+      </x:c>
+      <x:c r="I824" s="4" t="str">
+        <x:v>Q</x:v>
+      </x:c>
+      <x:c r="J824" s="4" t="str">
+        <x:v>Q</x:v>
+      </x:c>
+      <x:c r="K824" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L824" s="4" t="str">
+        <x:v>Q10,Q11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="825">
+      <x:c r="A825" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B825" s="4" t="str">
+        <x:v>Q04_01_H18</x:v>
+      </x:c>
+      <x:c r="C825" s="4" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="D825" s="4" t="str">
+        <x:v>君乐宝 益生菌发酵乳8／16联杯装</x:v>
+      </x:c>
+      <x:c r="E825" s="4" t="str">
+        <x:v>k</x:v>
+      </x:c>
+      <x:c r="F825" s="4" t="str"/>
+      <x:c r="G825" s="4" t="str">
+        <x:v>k</x:v>
+      </x:c>
+      <x:c r="H825" s="4" t="str">
+        <x:v>k</x:v>
+      </x:c>
+      <x:c r="I825" s="4" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="J825" s="4" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="K825" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L825" s="4" t="str">
+        <x:v>R10,R11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="826">
+      <x:c r="A826" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B826" s="4" t="str">
+        <x:v>Q04_01_H19</x:v>
+      </x:c>
+      <x:c r="C826" s="4" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D826" s="4" t="str">
+        <x:v>光明 益生菌风味发酵乳系列</x:v>
+      </x:c>
+      <x:c r="E826" s="4" t="str">
+        <x:v>l</x:v>
+      </x:c>
+      <x:c r="F826" s="4" t="str"/>
+      <x:c r="G826" s="4" t="str">
+        <x:v>l</x:v>
+      </x:c>
+      <x:c r="H826" s="4" t="str">
+        <x:v>l</x:v>
+      </x:c>
+      <x:c r="I826" s="4" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="J826" s="4" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="K826" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L826" s="4" t="str">
+        <x:v>S10,S11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="827">
+      <x:c r="A827" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B827" s="4" t="str">
+        <x:v>Q04_01_H20</x:v>
+      </x:c>
+      <x:c r="C827" s="4" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="D827" s="4" t="str">
+        <x:v>蒙牛 冠益乳利乐冠</x:v>
+      </x:c>
+      <x:c r="E827" s="4" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="F827" s="4" t="str"/>
+      <x:c r="G827" s="4" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="H827" s="4" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="I827" s="4" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="J827" s="4" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="K827" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L827" s="4" t="str">
+        <x:v>T10,T11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="828">
+      <x:c r="A828" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B828" s="4" t="str">
+        <x:v>Q04_01_H21</x:v>
+      </x:c>
+      <x:c r="C828" s="4" t="str">
+        <x:v>U</x:v>
+      </x:c>
+      <x:c r="D828" s="4" t="str">
+        <x:v>蒙牛 冠益乳免疫力瓶（健字号）</x:v>
+      </x:c>
+      <x:c r="E828" s="4" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="F828" s="4" t="str"/>
+      <x:c r="G828" s="4" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="H828" s="4" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="I828" s="4" t="str">
+        <x:v>U</x:v>
+      </x:c>
+      <x:c r="J828" s="4" t="str">
+        <x:v>U</x:v>
+      </x:c>
+      <x:c r="K828" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L828" s="4" t="str">
+        <x:v>U10,U11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="829">
+      <x:c r="A829" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B829" s="4" t="str">
+        <x:v>Q04_01_H22</x:v>
+      </x:c>
+      <x:c r="C829" s="4" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D829" s="4" t="str">
+        <x:v>光明 畅优系列</x:v>
+      </x:c>
+      <x:c r="E829" s="4" t="str">
+        <x:v>o</x:v>
+      </x:c>
+      <x:c r="F829" s="4" t="str"/>
+      <x:c r="G829" s="4" t="str">
+        <x:v>o</x:v>
+      </x:c>
+      <x:c r="H829" s="4" t="str">
+        <x:v>o</x:v>
+      </x:c>
+      <x:c r="I829" s="4" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="J829" s="4" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="K829" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L829" s="4" t="str">
+        <x:v>V10,V11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="830">
+      <x:c r="A830" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B830" s="4" t="str">
+        <x:v>Q04_01_H23</x:v>
+      </x:c>
+      <x:c r="C830" s="4" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="D830" s="4" t="str">
+        <x:v>伊利 益消系列</x:v>
+      </x:c>
+      <x:c r="E830" s="4" t="str">
+        <x:v>p</x:v>
+      </x:c>
+      <x:c r="F830" s="4" t="str"/>
+      <x:c r="G830" s="4" t="str">
+        <x:v>p</x:v>
+      </x:c>
+      <x:c r="H830" s="4" t="str">
+        <x:v>p</x:v>
+      </x:c>
+      <x:c r="I830" s="4" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="J830" s="4" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="K830" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L830" s="4" t="str">
+        <x:v>W10,W11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="831">
+      <x:c r="A831" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B831" s="4" t="str">
+        <x:v>Q04_01_H24</x:v>
+      </x:c>
+      <x:c r="C831" s="4" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D831" s="4" t="str">
+        <x:v>新希望 · 活润 活润轻食瓶／轻食杯</x:v>
+      </x:c>
+      <x:c r="E831" s="4" t="str">
+        <x:v>q</x:v>
+      </x:c>
+      <x:c r="F831" s="4" t="str"/>
+      <x:c r="G831" s="4" t="str">
+        <x:v>q</x:v>
+      </x:c>
+      <x:c r="H831" s="4" t="str">
+        <x:v>q</x:v>
+      </x:c>
+      <x:c r="I831" s="4" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="J831" s="4" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="K831" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L831" s="4" t="str">
+        <x:v>X10,X11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="832">
+      <x:c r="A832" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B832" s="4" t="str">
+        <x:v>Q04_01_H25</x:v>
+      </x:c>
+      <x:c r="C832" s="4" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D832" s="4" t="str">
+        <x:v>新希望 · 活润 活润晶球</x:v>
+      </x:c>
+      <x:c r="E832" s="4" t="str">
+        <x:v>r</x:v>
+      </x:c>
+      <x:c r="F832" s="4" t="str"/>
+      <x:c r="G832" s="4" t="str">
+        <x:v>r</x:v>
+      </x:c>
+      <x:c r="H832" s="4" t="str">
+        <x:v>r</x:v>
+      </x:c>
+      <x:c r="I832" s="4" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="J832" s="4" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="K832" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L832" s="4" t="str">
+        <x:v>Y10,Y11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="833">
+      <x:c r="A833" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B833" s="4" t="str">
+        <x:v>Q04_01_H26</x:v>
+      </x:c>
+      <x:c r="C833" s="4" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="D833" s="4" t="str">
+        <x:v>卡士 餐后一小时</x:v>
+      </x:c>
+      <x:c r="E833" s="4" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="F833" s="4" t="str"/>
+      <x:c r="G833" s="4" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="H833" s="4" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="I833" s="4" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="J833" s="4" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="K833" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L833" s="4" t="str">
+        <x:v>Z10,Z11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="834">
+      <x:c r="A834" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B834" s="4" t="str">
+        <x:v>Q04_01_H27</x:v>
+      </x:c>
+      <x:c r="C834" s="4" t="str">
+        <x:v>AA</x:v>
+      </x:c>
+      <x:c r="D834" s="4" t="str">
+        <x:v>简爱 顺畅配方酸奶</x:v>
+      </x:c>
+      <x:c r="E834" s="4" t="str">
+        <x:v>t</x:v>
+      </x:c>
+      <x:c r="F834" s="4" t="str"/>
+      <x:c r="G834" s="4" t="str">
+        <x:v>t</x:v>
+      </x:c>
+      <x:c r="H834" s="4" t="str">
+        <x:v>t</x:v>
+      </x:c>
+      <x:c r="I834" s="4" t="str">
+        <x:v>AA</x:v>
+      </x:c>
+      <x:c r="J834" s="4" t="str">
+        <x:v>AA</x:v>
+      </x:c>
+      <x:c r="K834" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L834" s="4" t="str">
+        <x:v>AA10,AA11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="835">
+      <x:c r="A835" s="4" t="str">
+        <x:v>Q04_01</x:v>
+      </x:c>
+      <x:c r="B835" s="4" t="str">
+        <x:v>Q04_01_H28</x:v>
+      </x:c>
+      <x:c r="C835" s="4" t="str">
+        <x:v>AB</x:v>
+      </x:c>
+      <x:c r="D835" s="4" t="str">
+        <x:v>卡士 007系列</x:v>
+      </x:c>
+      <x:c r="E835" s="4" t="str">
+        <x:v>u</x:v>
+      </x:c>
+      <x:c r="F835" s="4" t="str"/>
+      <x:c r="G835" s="4" t="str">
+        <x:v>u</x:v>
+      </x:c>
+      <x:c r="H835" s="4" t="str">
+        <x:v>u</x:v>
+      </x:c>
+      <x:c r="I835" s="4" t="str">
+        <x:v>AB</x:v>
+      </x:c>
+      <x:c r="J835" s="4" t="str">
+        <x:v>AB</x:v>
+      </x:c>
+      <x:c r="K835" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L835" s="4" t="str">
+        <x:v>AB10,AB11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="836">
+      <x:c r="A836" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B836" s="4" t="str">
+        <x:v>Q04_02_H2</x:v>
+      </x:c>
+      <x:c r="C836" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D836" s="4" t="str">
+        <x:v>Total</x:v>
+      </x:c>
+      <x:c r="E836" s="4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F836" s="4" t="str"/>
+      <x:c r="G836" s="4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H836" s="4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="I836" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J836" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K836" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L836" s="4" t="str">
+        <x:v>B88,B89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="837">
+      <x:c r="A837" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B837" s="4" t="str">
+        <x:v>Q04_02_H3</x:v>
+      </x:c>
+      <x:c r="C837" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D837" s="4" t="str">
+        <x:v>1~2线·有孩家庭</x:v>
+      </x:c>
+      <x:c r="E837" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F837" s="4" t="str"/>
+      <x:c r="G837" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H837" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="I837" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J837" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K837" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L837" s="4" t="str">
+        <x:v>C88,C89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="838">
+      <x:c r="A838" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B838" s="4" t="str">
+        <x:v>Q04_02_H4</x:v>
+      </x:c>
+      <x:c r="C838" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="D838" s="4" t="str">
+        <x:v>1~2线·其他家庭</x:v>
+      </x:c>
+      <x:c r="E838" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F838" s="4" t="str"/>
+      <x:c r="G838" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H838" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I838" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="J838" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="K838" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L838" s="4" t="str">
+        <x:v>D88,D89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="839">
+      <x:c r="A839" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B839" s="4" t="str">
+        <x:v>Q04_02_H5</x:v>
+      </x:c>
+      <x:c r="C839" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="D839" s="4" t="str">
+        <x:v>3线及以下</x:v>
+      </x:c>
+      <x:c r="E839" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="F839" s="4" t="str"/>
+      <x:c r="G839" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="H839" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="I839" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="J839" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="K839" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L839" s="4" t="str">
+        <x:v>E88,E89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="840">
+      <x:c r="A840" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B840" s="4" t="str">
+        <x:v>Q04_02_H6</x:v>
+      </x:c>
+      <x:c r="C840" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D840" s="4" t="str">
+        <x:v>低温用户</x:v>
+      </x:c>
+      <x:c r="E840" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="F840" s="4" t="str"/>
+      <x:c r="G840" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="H840" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="I840" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="J840" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="K840" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L840" s="4" t="str">
+        <x:v>F88,F89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="841">
+      <x:c r="A841" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B841" s="4" t="str">
+        <x:v>Q04_02_H7</x:v>
+      </x:c>
+      <x:c r="C841" s="4" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="D841" s="4" t="str">
+        <x:v>仅常温用户</x:v>
+      </x:c>
+      <x:c r="E841" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F841" s="4" t="str"/>
+      <x:c r="G841" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H841" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I841" s="4" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="J841" s="4" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="K841" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L841" s="4" t="str">
+        <x:v>G88,G89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="842">
+      <x:c r="A842" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B842" s="4" t="str">
+        <x:v>Q04_02_H8</x:v>
+      </x:c>
+      <x:c r="C842" s="4" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="D842" s="4" t="str">
+        <x:v>低温 Total</x:v>
+      </x:c>
+      <x:c r="E842" s="4" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="F842" s="4" t="str"/>
+      <x:c r="G842" s="4" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="H842" s="4" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="I842" s="4" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="J842" s="4" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="K842" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L842" s="4" t="str">
+        <x:v>H88,H89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="843">
+      <x:c r="A843" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B843" s="4" t="str">
+        <x:v>Q04_02_H9</x:v>
+      </x:c>
+      <x:c r="C843" s="4" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D843" s="4" t="str">
+        <x:v>1~2线·有孩家庭</x:v>
+      </x:c>
+      <x:c r="E843" s="4" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="F843" s="4" t="str"/>
+      <x:c r="G843" s="4" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="H843" s="4" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="I843" s="4" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="J843" s="4" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="K843" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L843" s="4" t="str">
+        <x:v>I88,I89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="844">
+      <x:c r="A844" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B844" s="4" t="str">
+        <x:v>Q04_02_H10</x:v>
+      </x:c>
+      <x:c r="C844" s="4" t="str">
+        <x:v>J</x:v>
+      </x:c>
+      <x:c r="D844" s="4" t="str">
+        <x:v>1~2线·其他家庭</x:v>
+      </x:c>
+      <x:c r="E844" s="4" t="str">
+        <x:v>c</x:v>
+      </x:c>
+      <x:c r="F844" s="4" t="str"/>
+      <x:c r="G844" s="4" t="str">
+        <x:v>c</x:v>
+      </x:c>
+      <x:c r="H844" s="4" t="str">
+        <x:v>c</x:v>
+      </x:c>
+      <x:c r="I844" s="4" t="str">
+        <x:v>J</x:v>
+      </x:c>
+      <x:c r="J844" s="4" t="str">
+        <x:v>J</x:v>
+      </x:c>
+      <x:c r="K844" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L844" s="4" t="str">
+        <x:v>J88,J89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="845">
+      <x:c r="A845" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B845" s="4" t="str">
+        <x:v>Q04_02_H11</x:v>
+      </x:c>
+      <x:c r="C845" s="4" t="str">
+        <x:v>K</x:v>
+      </x:c>
+      <x:c r="D845" s="4" t="str">
+        <x:v>3线及以下</x:v>
+      </x:c>
+      <x:c r="E845" s="4" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="F845" s="4" t="str"/>
+      <x:c r="G845" s="4" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="H845" s="4" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="I845" s="4" t="str">
+        <x:v>K</x:v>
+      </x:c>
+      <x:c r="J845" s="4" t="str">
+        <x:v>K</x:v>
+      </x:c>
+      <x:c r="K845" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L845" s="4" t="str">
+        <x:v>K88,K89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="846">
+      <x:c r="A846" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B846" s="4" t="str">
+        <x:v>Q04_02_H12</x:v>
+      </x:c>
+      <x:c r="C846" s="4" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D846" s="4" t="str">
+        <x:v>L1 忠诚</x:v>
+      </x:c>
+      <x:c r="E846" s="4" t="str">
+        <x:v>e</x:v>
+      </x:c>
+      <x:c r="F846" s="4" t="str"/>
+      <x:c r="G846" s="4" t="str">
+        <x:v>e</x:v>
+      </x:c>
+      <x:c r="H846" s="4" t="str">
+        <x:v>e</x:v>
+      </x:c>
+      <x:c r="I846" s="4" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="J846" s="4" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="K846" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L846" s="4" t="str">
+        <x:v>L88,L89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="847">
+      <x:c r="A847" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B847" s="4" t="str">
+        <x:v>Q04_02_H13</x:v>
+      </x:c>
+      <x:c r="C847" s="4" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D847" s="4" t="str">
+        <x:v>L2 复购</x:v>
+      </x:c>
+      <x:c r="E847" s="4" t="str">
+        <x:v>f</x:v>
+      </x:c>
+      <x:c r="F847" s="4" t="str"/>
+      <x:c r="G847" s="4" t="str">
+        <x:v>f</x:v>
+      </x:c>
+      <x:c r="H847" s="4" t="str">
+        <x:v>f</x:v>
+      </x:c>
+      <x:c r="I847" s="4" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="J847" s="4" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="K847" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L847" s="4" t="str">
+        <x:v>M88,M89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="848">
+      <x:c r="A848" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B848" s="4" t="str">
+        <x:v>Q04_02_H14</x:v>
+      </x:c>
+      <x:c r="C848" s="4" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="D848" s="4" t="str">
+        <x:v>L3 试用</x:v>
+      </x:c>
+      <x:c r="E848" s="4" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="F848" s="4" t="str"/>
+      <x:c r="G848" s="4" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="H848" s="4" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="I848" s="4" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="J848" s="4" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="K848" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L848" s="4" t="str">
+        <x:v>N88,N89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="849">
+      <x:c r="A849" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B849" s="4" t="str">
+        <x:v>Q04_02_H15</x:v>
+      </x:c>
+      <x:c r="C849" s="4" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="D849" s="4" t="str">
+        <x:v>L4 错配</x:v>
+      </x:c>
+      <x:c r="E849" s="4" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="F849" s="4" t="str"/>
+      <x:c r="G849" s="4" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="H849" s="4" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="I849" s="4" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="J849" s="4" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="K849" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L849" s="4" t="str">
+        <x:v>O88,O89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="850">
+      <x:c r="A850" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B850" s="4" t="str">
+        <x:v>Q04_02_H16</x:v>
+      </x:c>
+      <x:c r="C850" s="4" t="str">
+        <x:v>P</x:v>
+      </x:c>
+      <x:c r="D850" s="4" t="str">
+        <x:v>L5 未买益生菌</x:v>
+      </x:c>
+      <x:c r="E850" s="4" t="str">
+        <x:v>i</x:v>
+      </x:c>
+      <x:c r="F850" s="4" t="str"/>
+      <x:c r="G850" s="4" t="str">
+        <x:v>i</x:v>
+      </x:c>
+      <x:c r="H850" s="4" t="str">
+        <x:v>i</x:v>
+      </x:c>
+      <x:c r="I850" s="4" t="str">
+        <x:v>P</x:v>
+      </x:c>
+      <x:c r="J850" s="4" t="str">
+        <x:v>P</x:v>
+      </x:c>
+      <x:c r="K850" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L850" s="4" t="str">
+        <x:v>P88,P89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="851">
+      <x:c r="A851" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B851" s="4" t="str">
+        <x:v>Q04_02_H17</x:v>
+      </x:c>
+      <x:c r="C851" s="4" t="str">
+        <x:v>Q</x:v>
+      </x:c>
+      <x:c r="D851" s="4" t="str">
+        <x:v>伊利 畅轻利乐冠系列</x:v>
+      </x:c>
+      <x:c r="E851" s="4" t="str">
+        <x:v>j</x:v>
+      </x:c>
+      <x:c r="F851" s="4" t="str"/>
+      <x:c r="G851" s="4" t="str">
+        <x:v>j</x:v>
+      </x:c>
+      <x:c r="H851" s="4" t="str">
+        <x:v>j</x:v>
+      </x:c>
+      <x:c r="I851" s="4" t="str">
+        <x:v>Q</x:v>
+      </x:c>
+      <x:c r="J851" s="4" t="str">
+        <x:v>Q</x:v>
+      </x:c>
+      <x:c r="K851" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L851" s="4" t="str">
+        <x:v>Q88,Q89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="852">
+      <x:c r="A852" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B852" s="4" t="str">
+        <x:v>Q04_02_H18</x:v>
+      </x:c>
+      <x:c r="C852" s="4" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="D852" s="4" t="str">
+        <x:v>君乐宝 益生菌发酵乳8／16联杯装</x:v>
+      </x:c>
+      <x:c r="E852" s="4" t="str">
+        <x:v>k</x:v>
+      </x:c>
+      <x:c r="F852" s="4" t="str"/>
+      <x:c r="G852" s="4" t="str">
+        <x:v>k</x:v>
+      </x:c>
+      <x:c r="H852" s="4" t="str">
+        <x:v>k</x:v>
+      </x:c>
+      <x:c r="I852" s="4" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="J852" s="4" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="K852" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L852" s="4" t="str">
+        <x:v>R88,R89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="853">
+      <x:c r="A853" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B853" s="4" t="str">
+        <x:v>Q04_02_H19</x:v>
+      </x:c>
+      <x:c r="C853" s="4" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D853" s="4" t="str">
+        <x:v>光明 益生菌风味发酵乳系列</x:v>
+      </x:c>
+      <x:c r="E853" s="4" t="str">
+        <x:v>l</x:v>
+      </x:c>
+      <x:c r="F853" s="4" t="str"/>
+      <x:c r="G853" s="4" t="str">
+        <x:v>l</x:v>
+      </x:c>
+      <x:c r="H853" s="4" t="str">
+        <x:v>l</x:v>
+      </x:c>
+      <x:c r="I853" s="4" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="J853" s="4" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="K853" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L853" s="4" t="str">
+        <x:v>S88,S89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="854">
+      <x:c r="A854" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B854" s="4" t="str">
+        <x:v>Q04_02_H20</x:v>
+      </x:c>
+      <x:c r="C854" s="4" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="D854" s="4" t="str">
+        <x:v>蒙牛 冠益乳利乐冠</x:v>
+      </x:c>
+      <x:c r="E854" s="4" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="F854" s="4" t="str"/>
+      <x:c r="G854" s="4" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="H854" s="4" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="I854" s="4" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="J854" s="4" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="K854" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L854" s="4" t="str">
+        <x:v>T88,T89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="855">
+      <x:c r="A855" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B855" s="4" t="str">
+        <x:v>Q04_02_H21</x:v>
+      </x:c>
+      <x:c r="C855" s="4" t="str">
+        <x:v>U</x:v>
+      </x:c>
+      <x:c r="D855" s="4" t="str">
+        <x:v>蒙牛 冠益乳免疫力瓶（健字号）</x:v>
+      </x:c>
+      <x:c r="E855" s="4" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="F855" s="4" t="str"/>
+      <x:c r="G855" s="4" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="H855" s="4" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="I855" s="4" t="str">
+        <x:v>U</x:v>
+      </x:c>
+      <x:c r="J855" s="4" t="str">
+        <x:v>U</x:v>
+      </x:c>
+      <x:c r="K855" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L855" s="4" t="str">
+        <x:v>U88,U89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="856">
+      <x:c r="A856" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B856" s="4" t="str">
+        <x:v>Q04_02_H22</x:v>
+      </x:c>
+      <x:c r="C856" s="4" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D856" s="4" t="str">
+        <x:v>光明 畅优系列</x:v>
+      </x:c>
+      <x:c r="E856" s="4" t="str">
+        <x:v>o</x:v>
+      </x:c>
+      <x:c r="F856" s="4" t="str"/>
+      <x:c r="G856" s="4" t="str">
+        <x:v>o</x:v>
+      </x:c>
+      <x:c r="H856" s="4" t="str">
+        <x:v>o</x:v>
+      </x:c>
+      <x:c r="I856" s="4" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="J856" s="4" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="K856" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L856" s="4" t="str">
+        <x:v>V88,V89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="857">
+      <x:c r="A857" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B857" s="4" t="str">
+        <x:v>Q04_02_H23</x:v>
+      </x:c>
+      <x:c r="C857" s="4" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="D857" s="4" t="str">
+        <x:v>伊利 益消系列</x:v>
+      </x:c>
+      <x:c r="E857" s="4" t="str">
+        <x:v>p</x:v>
+      </x:c>
+      <x:c r="F857" s="4" t="str"/>
+      <x:c r="G857" s="4" t="str">
+        <x:v>p</x:v>
+      </x:c>
+      <x:c r="H857" s="4" t="str">
+        <x:v>p</x:v>
+      </x:c>
+      <x:c r="I857" s="4" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="J857" s="4" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="K857" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L857" s="4" t="str">
+        <x:v>W88,W89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="858">
+      <x:c r="A858" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B858" s="4" t="str">
+        <x:v>Q04_02_H24</x:v>
+      </x:c>
+      <x:c r="C858" s="4" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D858" s="4" t="str">
+        <x:v>新希望 · 活润 活润轻食瓶／轻食杯</x:v>
+      </x:c>
+      <x:c r="E858" s="4" t="str">
+        <x:v>q</x:v>
+      </x:c>
+      <x:c r="F858" s="4" t="str"/>
+      <x:c r="G858" s="4" t="str">
+        <x:v>q</x:v>
+      </x:c>
+      <x:c r="H858" s="4" t="str">
+        <x:v>q</x:v>
+      </x:c>
+      <x:c r="I858" s="4" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="J858" s="4" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="K858" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L858" s="4" t="str">
+        <x:v>X88,X89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="859">
+      <x:c r="A859" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B859" s="4" t="str">
+        <x:v>Q04_02_H25</x:v>
+      </x:c>
+      <x:c r="C859" s="4" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D859" s="4" t="str">
+        <x:v>新希望 · 活润 活润晶球</x:v>
+      </x:c>
+      <x:c r="E859" s="4" t="str">
+        <x:v>r</x:v>
+      </x:c>
+      <x:c r="F859" s="4" t="str"/>
+      <x:c r="G859" s="4" t="str">
+        <x:v>r</x:v>
+      </x:c>
+      <x:c r="H859" s="4" t="str">
+        <x:v>r</x:v>
+      </x:c>
+      <x:c r="I859" s="4" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="J859" s="4" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="K859" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L859" s="4" t="str">
+        <x:v>Y88,Y89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="860">
+      <x:c r="A860" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B860" s="4" t="str">
+        <x:v>Q04_02_H26</x:v>
+      </x:c>
+      <x:c r="C860" s="4" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="D860" s="4" t="str">
+        <x:v>卡士 餐后一小时</x:v>
+      </x:c>
+      <x:c r="E860" s="4" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="F860" s="4" t="str"/>
+      <x:c r="G860" s="4" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="H860" s="4" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="I860" s="4" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="J860" s="4" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="K860" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L860" s="4" t="str">
+        <x:v>Z88,Z89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="861">
+      <x:c r="A861" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B861" s="4" t="str">
+        <x:v>Q04_02_H27</x:v>
+      </x:c>
+      <x:c r="C861" s="4" t="str">
+        <x:v>AA</x:v>
+      </x:c>
+      <x:c r="D861" s="4" t="str">
+        <x:v>简爱 顺畅配方酸奶</x:v>
+      </x:c>
+      <x:c r="E861" s="4" t="str">
+        <x:v>t</x:v>
+      </x:c>
+      <x:c r="F861" s="4" t="str"/>
+      <x:c r="G861" s="4" t="str">
+        <x:v>t</x:v>
+      </x:c>
+      <x:c r="H861" s="4" t="str">
+        <x:v>t</x:v>
+      </x:c>
+      <x:c r="I861" s="4" t="str">
+        <x:v>AA</x:v>
+      </x:c>
+      <x:c r="J861" s="4" t="str">
+        <x:v>AA</x:v>
+      </x:c>
+      <x:c r="K861" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L861" s="4" t="str">
+        <x:v>AA88,AA89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="862">
+      <x:c r="A862" s="4" t="str">
+        <x:v>Q04_02</x:v>
+      </x:c>
+      <x:c r="B862" s="4" t="str">
+        <x:v>Q04_02_H28</x:v>
+      </x:c>
+      <x:c r="C862" s="4" t="str">
+        <x:v>AB</x:v>
+      </x:c>
+      <x:c r="D862" s="4" t="str">
+        <x:v>卡士 007系列</x:v>
+      </x:c>
+      <x:c r="E862" s="4" t="str">
+        <x:v>u</x:v>
+      </x:c>
+      <x:c r="F862" s="4" t="str"/>
+      <x:c r="G862" s="4" t="str">
+        <x:v>u</x:v>
+      </x:c>
+      <x:c r="H862" s="4" t="str">
+        <x:v>u</x:v>
+      </x:c>
+      <x:c r="I862" s="4" t="str">
+        <x:v>AB</x:v>
+      </x:c>
+      <x:c r="J862" s="4" t="str">
+        <x:v>AB</x:v>
+      </x:c>
+      <x:c r="K862" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L862" s="4" t="str">
+        <x:v>AB88,AB89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="863">
+      <x:c r="A863" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B863" s="4" t="str">
+        <x:v>Q04_03_H2</x:v>
+      </x:c>
+      <x:c r="C863" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D863" s="4" t="str">
+        <x:v>Total</x:v>
+      </x:c>
+      <x:c r="E863" s="4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F863" s="4" t="str"/>
+      <x:c r="G863" s="4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H863" s="4" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="I863" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J863" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K863" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L863" s="4" t="str">
+        <x:v>B620,B621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="864">
+      <x:c r="A864" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B864" s="4" t="str">
+        <x:v>Q04_03_H3</x:v>
+      </x:c>
+      <x:c r="C864" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D864" s="4" t="str">
+        <x:v>1~2线·有孩家庭</x:v>
+      </x:c>
+      <x:c r="E864" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F864" s="4" t="str"/>
+      <x:c r="G864" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H864" s="4" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="I864" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J864" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K864" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L864" s="4" t="str">
+        <x:v>C620,C621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="865">
+      <x:c r="A865" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B865" s="4" t="str">
+        <x:v>Q04_03_H4</x:v>
+      </x:c>
+      <x:c r="C865" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="D865" s="4" t="str">
+        <x:v>1~2线·其他家庭</x:v>
+      </x:c>
+      <x:c r="E865" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F865" s="4" t="str"/>
+      <x:c r="G865" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H865" s="4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I865" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="J865" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="K865" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L865" s="4" t="str">
+        <x:v>D620,D621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="866">
+      <x:c r="A866" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B866" s="4" t="str">
+        <x:v>Q04_03_H5</x:v>
+      </x:c>
+      <x:c r="C866" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="D866" s="4" t="str">
+        <x:v>3线及以下</x:v>
+      </x:c>
+      <x:c r="E866" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="F866" s="4" t="str"/>
+      <x:c r="G866" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="H866" s="4" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="I866" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="J866" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="K866" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L866" s="4" t="str">
+        <x:v>E620,E621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="867">
+      <x:c r="A867" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B867" s="4" t="str">
+        <x:v>Q04_03_H6</x:v>
+      </x:c>
+      <x:c r="C867" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D867" s="4" t="str">
+        <x:v>低温用户</x:v>
+      </x:c>
+      <x:c r="E867" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="F867" s="4" t="str"/>
+      <x:c r="G867" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="H867" s="4" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="I867" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="J867" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="K867" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L867" s="4" t="str">
+        <x:v>F620,F621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="868">
+      <x:c r="A868" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B868" s="4" t="str">
+        <x:v>Q04_03_H7</x:v>
+      </x:c>
+      <x:c r="C868" s="4" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="D868" s="4" t="str">
+        <x:v>仅常温用户</x:v>
+      </x:c>
+      <x:c r="E868" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F868" s="4" t="str"/>
+      <x:c r="G868" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H868" s="4" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I868" s="4" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="J868" s="4" t="str">
+        <x:v>G</x:v>
+      </x:c>
+      <x:c r="K868" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L868" s="4" t="str">
+        <x:v>G620,G621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="869">
+      <x:c r="A869" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B869" s="4" t="str">
+        <x:v>Q04_03_H8</x:v>
+      </x:c>
+      <x:c r="C869" s="4" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="D869" s="4" t="str">
+        <x:v>低温 Total</x:v>
+      </x:c>
+      <x:c r="E869" s="4" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="F869" s="4" t="str"/>
+      <x:c r="G869" s="4" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="H869" s="4" t="str">
+        <x:v>a</x:v>
+      </x:c>
+      <x:c r="I869" s="4" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="J869" s="4" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="K869" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L869" s="4" t="str">
+        <x:v>H620,H621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="870">
+      <x:c r="A870" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B870" s="4" t="str">
+        <x:v>Q04_03_H9</x:v>
+      </x:c>
+      <x:c r="C870" s="4" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="D870" s="4" t="str">
+        <x:v>1~2线·有孩家庭</x:v>
+      </x:c>
+      <x:c r="E870" s="4" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="F870" s="4" t="str"/>
+      <x:c r="G870" s="4" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="H870" s="4" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="I870" s="4" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="J870" s="4" t="str">
+        <x:v>I</x:v>
+      </x:c>
+      <x:c r="K870" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L870" s="4" t="str">
+        <x:v>I620,I621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="871">
+      <x:c r="A871" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B871" s="4" t="str">
+        <x:v>Q04_03_H10</x:v>
+      </x:c>
+      <x:c r="C871" s="4" t="str">
+        <x:v>J</x:v>
+      </x:c>
+      <x:c r="D871" s="4" t="str">
+        <x:v>1~2线·其他家庭</x:v>
+      </x:c>
+      <x:c r="E871" s="4" t="str">
+        <x:v>c</x:v>
+      </x:c>
+      <x:c r="F871" s="4" t="str"/>
+      <x:c r="G871" s="4" t="str">
+        <x:v>c</x:v>
+      </x:c>
+      <x:c r="H871" s="4" t="str">
+        <x:v>c</x:v>
+      </x:c>
+      <x:c r="I871" s="4" t="str">
+        <x:v>J</x:v>
+      </x:c>
+      <x:c r="J871" s="4" t="str">
+        <x:v>J</x:v>
+      </x:c>
+      <x:c r="K871" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L871" s="4" t="str">
+        <x:v>J620,J621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="872">
+      <x:c r="A872" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B872" s="4" t="str">
+        <x:v>Q04_03_H11</x:v>
+      </x:c>
+      <x:c r="C872" s="4" t="str">
+        <x:v>K</x:v>
+      </x:c>
+      <x:c r="D872" s="4" t="str">
+        <x:v>3线及以下</x:v>
+      </x:c>
+      <x:c r="E872" s="4" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="F872" s="4" t="str"/>
+      <x:c r="G872" s="4" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="H872" s="4" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="I872" s="4" t="str">
+        <x:v>K</x:v>
+      </x:c>
+      <x:c r="J872" s="4" t="str">
+        <x:v>K</x:v>
+      </x:c>
+      <x:c r="K872" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L872" s="4" t="str">
+        <x:v>K620,K621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="873">
+      <x:c r="A873" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B873" s="4" t="str">
+        <x:v>Q04_03_H12</x:v>
+      </x:c>
+      <x:c r="C873" s="4" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="D873" s="4" t="str">
+        <x:v>L1 忠诚</x:v>
+      </x:c>
+      <x:c r="E873" s="4" t="str">
+        <x:v>e</x:v>
+      </x:c>
+      <x:c r="F873" s="4" t="str"/>
+      <x:c r="G873" s="4" t="str">
+        <x:v>e</x:v>
+      </x:c>
+      <x:c r="H873" s="4" t="str">
+        <x:v>e</x:v>
+      </x:c>
+      <x:c r="I873" s="4" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="J873" s="4" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="K873" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L873" s="4" t="str">
+        <x:v>L620,L621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="874">
+      <x:c r="A874" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B874" s="4" t="str">
+        <x:v>Q04_03_H13</x:v>
+      </x:c>
+      <x:c r="C874" s="4" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="D874" s="4" t="str">
+        <x:v>L2 复购</x:v>
+      </x:c>
+      <x:c r="E874" s="4" t="str">
+        <x:v>f</x:v>
+      </x:c>
+      <x:c r="F874" s="4" t="str"/>
+      <x:c r="G874" s="4" t="str">
+        <x:v>f</x:v>
+      </x:c>
+      <x:c r="H874" s="4" t="str">
+        <x:v>f</x:v>
+      </x:c>
+      <x:c r="I874" s="4" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="J874" s="4" t="str">
+        <x:v>M</x:v>
+      </x:c>
+      <x:c r="K874" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L874" s="4" t="str">
+        <x:v>M620,M621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="875">
+      <x:c r="A875" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B875" s="4" t="str">
+        <x:v>Q04_03_H14</x:v>
+      </x:c>
+      <x:c r="C875" s="4" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="D875" s="4" t="str">
+        <x:v>L3 试用</x:v>
+      </x:c>
+      <x:c r="E875" s="4" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="F875" s="4" t="str"/>
+      <x:c r="G875" s="4" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="H875" s="4" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="I875" s="4" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="J875" s="4" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="K875" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L875" s="4" t="str">
+        <x:v>N620,N621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="876">
+      <x:c r="A876" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B876" s="4" t="str">
+        <x:v>Q04_03_H15</x:v>
+      </x:c>
+      <x:c r="C876" s="4" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="D876" s="4" t="str">
+        <x:v>L4 错配</x:v>
+      </x:c>
+      <x:c r="E876" s="4" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="F876" s="4" t="str"/>
+      <x:c r="G876" s="4" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="H876" s="4" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="I876" s="4" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="J876" s="4" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="K876" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L876" s="4" t="str">
+        <x:v>O620,O621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="877">
+      <x:c r="A877" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B877" s="4" t="str">
+        <x:v>Q04_03_H16</x:v>
+      </x:c>
+      <x:c r="C877" s="4" t="str">
+        <x:v>P</x:v>
+      </x:c>
+      <x:c r="D877" s="4" t="str">
+        <x:v>L5 未买益生菌</x:v>
+      </x:c>
+      <x:c r="E877" s="4" t="str">
+        <x:v>i</x:v>
+      </x:c>
+      <x:c r="F877" s="4" t="str"/>
+      <x:c r="G877" s="4" t="str">
+        <x:v>i</x:v>
+      </x:c>
+      <x:c r="H877" s="4" t="str">
+        <x:v>i</x:v>
+      </x:c>
+      <x:c r="I877" s="4" t="str">
+        <x:v>P</x:v>
+      </x:c>
+      <x:c r="J877" s="4" t="str">
+        <x:v>P</x:v>
+      </x:c>
+      <x:c r="K877" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L877" s="4" t="str">
+        <x:v>P620,P621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="878">
+      <x:c r="A878" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B878" s="4" t="str">
+        <x:v>Q04_03_H17</x:v>
+      </x:c>
+      <x:c r="C878" s="4" t="str">
+        <x:v>Q</x:v>
+      </x:c>
+      <x:c r="D878" s="4" t="str">
+        <x:v>伊利 畅轻利乐冠系列</x:v>
+      </x:c>
+      <x:c r="E878" s="4" t="str">
+        <x:v>j</x:v>
+      </x:c>
+      <x:c r="F878" s="4" t="str"/>
+      <x:c r="G878" s="4" t="str">
+        <x:v>j</x:v>
+      </x:c>
+      <x:c r="H878" s="4" t="str">
+        <x:v>j</x:v>
+      </x:c>
+      <x:c r="I878" s="4" t="str">
+        <x:v>Q</x:v>
+      </x:c>
+      <x:c r="J878" s="4" t="str">
+        <x:v>Q</x:v>
+      </x:c>
+      <x:c r="K878" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L878" s="4" t="str">
+        <x:v>Q620,Q621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="879">
+      <x:c r="A879" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B879" s="4" t="str">
+        <x:v>Q04_03_H18</x:v>
+      </x:c>
+      <x:c r="C879" s="4" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="D879" s="4" t="str">
+        <x:v>君乐宝 益生菌发酵乳8／16联杯装</x:v>
+      </x:c>
+      <x:c r="E879" s="4" t="str">
+        <x:v>k</x:v>
+      </x:c>
+      <x:c r="F879" s="4" t="str"/>
+      <x:c r="G879" s="4" t="str">
+        <x:v>k</x:v>
+      </x:c>
+      <x:c r="H879" s="4" t="str">
+        <x:v>k</x:v>
+      </x:c>
+      <x:c r="I879" s="4" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="J879" s="4" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="K879" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L879" s="4" t="str">
+        <x:v>R620,R621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="880">
+      <x:c r="A880" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B880" s="4" t="str">
+        <x:v>Q04_03_H19</x:v>
+      </x:c>
+      <x:c r="C880" s="4" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="D880" s="4" t="str">
+        <x:v>光明 益生菌风味发酵乳系列</x:v>
+      </x:c>
+      <x:c r="E880" s="4" t="str">
+        <x:v>l</x:v>
+      </x:c>
+      <x:c r="F880" s="4" t="str"/>
+      <x:c r="G880" s="4" t="str">
+        <x:v>l</x:v>
+      </x:c>
+      <x:c r="H880" s="4" t="str">
+        <x:v>l</x:v>
+      </x:c>
+      <x:c r="I880" s="4" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="J880" s="4" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="K880" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L880" s="4" t="str">
+        <x:v>S620,S621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="881">
+      <x:c r="A881" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B881" s="4" t="str">
+        <x:v>Q04_03_H20</x:v>
+      </x:c>
+      <x:c r="C881" s="4" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="D881" s="4" t="str">
+        <x:v>蒙牛 冠益乳利乐冠</x:v>
+      </x:c>
+      <x:c r="E881" s="4" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="F881" s="4" t="str"/>
+      <x:c r="G881" s="4" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="H881" s="4" t="str">
+        <x:v>m</x:v>
+      </x:c>
+      <x:c r="I881" s="4" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="J881" s="4" t="str">
+        <x:v>T</x:v>
+      </x:c>
+      <x:c r="K881" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L881" s="4" t="str">
+        <x:v>T620,T621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="882">
+      <x:c r="A882" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B882" s="4" t="str">
+        <x:v>Q04_03_H21</x:v>
+      </x:c>
+      <x:c r="C882" s="4" t="str">
+        <x:v>U</x:v>
+      </x:c>
+      <x:c r="D882" s="4" t="str">
+        <x:v>蒙牛 冠益乳免疫力瓶（健字号）</x:v>
+      </x:c>
+      <x:c r="E882" s="4" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="F882" s="4" t="str"/>
+      <x:c r="G882" s="4" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="H882" s="4" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="I882" s="4" t="str">
+        <x:v>U</x:v>
+      </x:c>
+      <x:c r="J882" s="4" t="str">
+        <x:v>U</x:v>
+      </x:c>
+      <x:c r="K882" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L882" s="4" t="str">
+        <x:v>U620,U621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="883">
+      <x:c r="A883" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B883" s="4" t="str">
+        <x:v>Q04_03_H22</x:v>
+      </x:c>
+      <x:c r="C883" s="4" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D883" s="4" t="str">
+        <x:v>光明 畅优系列</x:v>
+      </x:c>
+      <x:c r="E883" s="4" t="str">
+        <x:v>o</x:v>
+      </x:c>
+      <x:c r="F883" s="4" t="str"/>
+      <x:c r="G883" s="4" t="str">
+        <x:v>o</x:v>
+      </x:c>
+      <x:c r="H883" s="4" t="str">
+        <x:v>o</x:v>
+      </x:c>
+      <x:c r="I883" s="4" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="J883" s="4" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="K883" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L883" s="4" t="str">
+        <x:v>V620,V621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="884">
+      <x:c r="A884" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B884" s="4" t="str">
+        <x:v>Q04_03_H23</x:v>
+      </x:c>
+      <x:c r="C884" s="4" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="D884" s="4" t="str">
+        <x:v>伊利 益消系列</x:v>
+      </x:c>
+      <x:c r="E884" s="4" t="str">
+        <x:v>p</x:v>
+      </x:c>
+      <x:c r="F884" s="4" t="str"/>
+      <x:c r="G884" s="4" t="str">
+        <x:v>p</x:v>
+      </x:c>
+      <x:c r="H884" s="4" t="str">
+        <x:v>p</x:v>
+      </x:c>
+      <x:c r="I884" s="4" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="J884" s="4" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="K884" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L884" s="4" t="str">
+        <x:v>W620,W621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="885">
+      <x:c r="A885" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B885" s="4" t="str">
+        <x:v>Q04_03_H24</x:v>
+      </x:c>
+      <x:c r="C885" s="4" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D885" s="4" t="str">
+        <x:v>新希望 · 活润 活润轻食瓶／轻食杯</x:v>
+      </x:c>
+      <x:c r="E885" s="4" t="str">
+        <x:v>q</x:v>
+      </x:c>
+      <x:c r="F885" s="4" t="str"/>
+      <x:c r="G885" s="4" t="str">
+        <x:v>q</x:v>
+      </x:c>
+      <x:c r="H885" s="4" t="str">
+        <x:v>q</x:v>
+      </x:c>
+      <x:c r="I885" s="4" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="J885" s="4" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="K885" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L885" s="4" t="str">
+        <x:v>X620,X621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="886">
+      <x:c r="A886" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B886" s="4" t="str">
+        <x:v>Q04_03_H25</x:v>
+      </x:c>
+      <x:c r="C886" s="4" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D886" s="4" t="str">
+        <x:v>新希望 · 活润 活润晶球</x:v>
+      </x:c>
+      <x:c r="E886" s="4" t="str">
+        <x:v>r</x:v>
+      </x:c>
+      <x:c r="F886" s="4" t="str"/>
+      <x:c r="G886" s="4" t="str">
+        <x:v>r</x:v>
+      </x:c>
+      <x:c r="H886" s="4" t="str">
+        <x:v>r</x:v>
+      </x:c>
+      <x:c r="I886" s="4" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="J886" s="4" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="K886" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L886" s="4" t="str">
+        <x:v>Y620,Y621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="887">
+      <x:c r="A887" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B887" s="4" t="str">
+        <x:v>Q04_03_H26</x:v>
+      </x:c>
+      <x:c r="C887" s="4" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="D887" s="4" t="str">
+        <x:v>卡士 餐后一小时</x:v>
+      </x:c>
+      <x:c r="E887" s="4" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="F887" s="4" t="str"/>
+      <x:c r="G887" s="4" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="H887" s="4" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="I887" s="4" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="J887" s="4" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="K887" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L887" s="4" t="str">
+        <x:v>Z620,Z621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="888">
+      <x:c r="A888" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B888" s="4" t="str">
+        <x:v>Q04_03_H27</x:v>
+      </x:c>
+      <x:c r="C888" s="4" t="str">
+        <x:v>AA</x:v>
+      </x:c>
+      <x:c r="D888" s="4" t="str">
+        <x:v>简爱 顺畅配方酸奶</x:v>
+      </x:c>
+      <x:c r="E888" s="4" t="str">
+        <x:v>t</x:v>
+      </x:c>
+      <x:c r="F888" s="4" t="str"/>
+      <x:c r="G888" s="4" t="str">
+        <x:v>t</x:v>
+      </x:c>
+      <x:c r="H888" s="4" t="str">
+        <x:v>t</x:v>
+      </x:c>
+      <x:c r="I888" s="4" t="str">
+        <x:v>AA</x:v>
+      </x:c>
+      <x:c r="J888" s="4" t="str">
+        <x:v>AA</x:v>
+      </x:c>
+      <x:c r="K888" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L888" s="4" t="str">
+        <x:v>AA620,AA621</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="889">
+      <x:c r="A889" s="4" t="str">
+        <x:v>Q04_03</x:v>
+      </x:c>
+      <x:c r="B889" s="4" t="str">
+        <x:v>Q04_03_H28</x:v>
+      </x:c>
+      <x:c r="C889" s="4" t="str">
+        <x:v>AB</x:v>
+      </x:c>
+      <x:c r="D889" s="4" t="str">
+        <x:v>卡士 007系列</x:v>
+      </x:c>
+      <x:c r="E889" s="4" t="str">
+        <x:v>u</x:v>
+      </x:c>
+      <x:c r="F889" s="4" t="str"/>
+      <x:c r="G889" s="4" t="str">
+        <x:v>u</x:v>
+      </x:c>
+      <x:c r="H889" s="4" t="str">
+        <x:v>u</x:v>
+      </x:c>
+      <x:c r="I889" s="4" t="str">
+        <x:v>AB</x:v>
+      </x:c>
+      <x:c r="J889" s="4" t="str">
+        <x:v>AB</x:v>
+      </x:c>
+      <x:c r="K889" s="4" t="str">
+        <x:v>mapped</x:v>
+      </x:c>
+      <x:c r="L889" s="4" t="str">
+        <x:v>AB620,AB621</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -33596,20 +36512,14 @@
       <x:c r="O65" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P65" s="4" t="n">
-        <x:v>0.094</x:v>
-      </x:c>
-      <x:c r="Q65" s="4" t="str">
-        <x:v>B14</x:v>
-      </x:c>
+      <x:c r="P65" s="4" t="str"/>
+      <x:c r="Q65" s="4" t="str"/>
       <x:c r="R65" s="4" t="str">
         <x:v>following_row</x:v>
       </x:c>
-      <x:c r="S65" s="4" t="str">
-        <x:v>unknown:0,unknown:.,unknown:0,unknown:9,unknown:4</x:v>
-      </x:c>
+      <x:c r="S65" s="4" t="str"/>
       <x:c r="T65" s="4" t="str">
-        <x:v>unresolved</x:v>
+        <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="U65" s="4" t="str">
         <x:v>base</x:v>
@@ -33657,20 +36567,14 @@
       <x:c r="O66" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P66" s="4" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="Q66" s="4" t="str">
-        <x:v>B15</x:v>
-      </x:c>
+      <x:c r="P66" s="4" t="str"/>
+      <x:c r="Q66" s="4" t="str"/>
       <x:c r="R66" s="4" t="str">
         <x:v>following_row</x:v>
       </x:c>
-      <x:c r="S66" s="4" t="str">
-        <x:v>Q03_01_H5</x:v>
-      </x:c>
+      <x:c r="S66" s="4" t="str"/>
       <x:c r="T66" s="4" t="str">
-        <x:v>mapped</x:v>
+        <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="U66" s="4" t="str">
         <x:v>data</x:v>
@@ -33779,20 +36683,14 @@
       <x:c r="O68" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P68" s="4" t="n">
-        <x:v>0.094</x:v>
-      </x:c>
-      <x:c r="Q68" s="4" t="str">
-        <x:v>B92</x:v>
-      </x:c>
+      <x:c r="P68" s="4" t="str"/>
+      <x:c r="Q68" s="4" t="str"/>
       <x:c r="R68" s="4" t="str">
         <x:v>following_row</x:v>
       </x:c>
-      <x:c r="S68" s="4" t="str">
-        <x:v>unknown:0,unknown:.,unknown:0,unknown:9,unknown:4</x:v>
-      </x:c>
+      <x:c r="S68" s="4" t="str"/>
       <x:c r="T68" s="4" t="str">
-        <x:v>unresolved</x:v>
+        <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="U68" s="4" t="str">
         <x:v>base</x:v>
@@ -33840,20 +36738,14 @@
       <x:c r="O69" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P69" s="4" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="Q69" s="4" t="str">
-        <x:v>B93</x:v>
-      </x:c>
+      <x:c r="P69" s="4" t="str"/>
+      <x:c r="Q69" s="4" t="str"/>
       <x:c r="R69" s="4" t="str">
         <x:v>following_row</x:v>
       </x:c>
-      <x:c r="S69" s="4" t="str">
-        <x:v>Q03_02_H5</x:v>
-      </x:c>
+      <x:c r="S69" s="4" t="str"/>
       <x:c r="T69" s="4" t="str">
-        <x:v>mapped</x:v>
+        <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="U69" s="4" t="str">
         <x:v>data</x:v>
@@ -33962,20 +36854,14 @@
       <x:c r="O71" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P71" s="4" t="n">
-        <x:v>0.25</x:v>
-      </x:c>
-      <x:c r="Q71" s="4" t="str">
-        <x:v>B624</x:v>
-      </x:c>
+      <x:c r="P71" s="4" t="str"/>
+      <x:c r="Q71" s="4" t="str"/>
       <x:c r="R71" s="4" t="str">
         <x:v>following_row</x:v>
       </x:c>
-      <x:c r="S71" s="4" t="str">
-        <x:v>unknown:0,unknown:.,unknown:2,unknown:5</x:v>
-      </x:c>
+      <x:c r="S71" s="4" t="str"/>
       <x:c r="T71" s="4" t="str">
-        <x:v>unresolved</x:v>
+        <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="U71" s="4" t="str">
         <x:v>base</x:v>
@@ -34023,20 +36909,14 @@
       <x:c r="O72" s="6" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="P72" s="4" t="str">
-        <x:v>DF</x:v>
-      </x:c>
-      <x:c r="Q72" s="4" t="str">
-        <x:v>B625</x:v>
-      </x:c>
+      <x:c r="P72" s="4" t="str"/>
+      <x:c r="Q72" s="4" t="str"/>
       <x:c r="R72" s="4" t="str">
         <x:v>following_row</x:v>
       </x:c>
-      <x:c r="S72" s="4" t="str">
-        <x:v>Q03_03_H5,Q03_03_H7</x:v>
-      </x:c>
+      <x:c r="S72" s="4" t="str"/>
       <x:c r="T72" s="4" t="str">
-        <x:v>mapped</x:v>
+        <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="U72" s="4" t="str">
         <x:v>data</x:v>

</xml_diff>

<commit_message>
fix: align table boundaries and strengthen detail prompt
</commit_message>
<xml_diff>
--- a/outputs/golden_annotation_final/Golden_Annotation_Final.xlsx
+++ b/outputs/golden_annotation_final/Golden_Annotation_Final.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_Me" sheetId="1" r:id="R2eb905db17b74f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workbook_Info" sheetId="2" r:id="Rbaf372ce76854665"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet_Annotation" sheetId="3" r:id="Rc71344d428cc40cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_Annotation" sheetId="4" r:id="R253e369303e34583"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Header_Annotation" sheetId="5" r:id="R90e0582164b747e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cell_Truth" sheetId="6" r:id="R7d37dffff06f4522"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Significance_Parsing_Cases" sheetId="7" r:id="R140100a1467b4b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_Me" sheetId="1" r:id="Rbf0dd65d9d02495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workbook_Info" sheetId="2" r:id="R73182fca2873494b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet_Annotation" sheetId="3" r:id="Rae9503db6c38474e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_Annotation" sheetId="4" r:id="R0b84efd9f5a24303"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Header_Annotation" sheetId="5" r:id="Rb79ce2fab81b44cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cell_Truth" sheetId="6" r:id="R1a287dada75542a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Significance_Parsing_Cases" sheetId="7" r:id="R389b4a3bc2f5433a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2538,7 +2538,7 @@
         <x:v>Quantum</x:v>
       </x:c>
       <x:c r="F23" s="4" t="str">
-        <x:v>A1:AB78</x:v>
+        <x:v>A2:AB77</x:v>
       </x:c>
       <x:c r="G23" s="4" t="str">
         <x:v>S1a</x:v>
@@ -2550,7 +2550,7 @@
         <x:v>S1a.请问您目前长期居住在哪个城市？（单选）</x:v>
       </x:c>
       <x:c r="J23" s="4" t="str">
-        <x:v>1:2</x:v>
+        <x:v>2:3</x:v>
       </x:c>
       <x:c r="K23" s="4" t="str">
         <x:v>10,11</x:v>
@@ -2562,7 +2562,7 @@
         <x:v>14:74</x:v>
       </x:c>
       <x:c r="N23" s="4" t="str">
-        <x:v>77:78</x:v>
+        <x:v>77:77</x:v>
       </x:c>
       <x:c r="O23" s="4" t="str">
         <x:v>percentage</x:v>
@@ -2616,7 +2616,7 @@
         <x:v>Quantum</x:v>
       </x:c>
       <x:c r="F24" s="4" t="str">
-        <x:v>A79:AB610</x:v>
+        <x:v>A80:AB609</x:v>
       </x:c>
       <x:c r="G24" s="4" t="str">
         <x:v>S1b</x:v>
@@ -2628,7 +2628,7 @@
         <x:v>S1b.请问您目前长期居住在哪个城市？（单选）</x:v>
       </x:c>
       <x:c r="J24" s="4" t="str">
-        <x:v>79:80</x:v>
+        <x:v>80:81</x:v>
       </x:c>
       <x:c r="K24" s="4" t="str">
         <x:v>88,89</x:v>
@@ -2640,7 +2640,7 @@
         <x:v>92:607</x:v>
       </x:c>
       <x:c r="N24" s="4" t="str">
-        <x:v>609:610</x:v>
+        <x:v>609:609</x:v>
       </x:c>
       <x:c r="O24" s="4" t="str">
         <x:v>percentage</x:v>
@@ -2694,7 +2694,7 @@
         <x:v>Quantum</x:v>
       </x:c>
       <x:c r="F25" s="4" t="str">
-        <x:v>A611:AB638</x:v>
+        <x:v>A612:AB637</x:v>
       </x:c>
       <x:c r="G25" s="4" t="str">
         <x:v>Tier</x:v>
@@ -2706,7 +2706,7 @@
         <x:v>Tier.Tier</x:v>
       </x:c>
       <x:c r="J25" s="4" t="str">
-        <x:v>611:612</x:v>
+        <x:v>612:613</x:v>
       </x:c>
       <x:c r="K25" s="4" t="str">
         <x:v>620,621</x:v>
@@ -2718,7 +2718,7 @@
         <x:v>624:635</x:v>
       </x:c>
       <x:c r="N25" s="4" t="str">
-        <x:v>637:638</x:v>
+        <x:v>637:637</x:v>
       </x:c>
       <x:c r="O25" s="4" t="str">
         <x:v>percentage</x:v>
@@ -2772,7 +2772,7 @@
         <x:v>Quantum</x:v>
       </x:c>
       <x:c r="F26" s="4" t="str">
-        <x:v>A1:AB78</x:v>
+        <x:v>A2:AB77</x:v>
       </x:c>
       <x:c r="G26" s="4" t="str">
         <x:v>S1a</x:v>
@@ -2784,7 +2784,7 @@
         <x:v>S1a.请问您目前长期居住在哪个城市？（单选）</x:v>
       </x:c>
       <x:c r="J26" s="4" t="str">
-        <x:v>1:2</x:v>
+        <x:v>2:3</x:v>
       </x:c>
       <x:c r="K26" s="4" t="str">
         <x:v>10,11</x:v>
@@ -2796,7 +2796,7 @@
         <x:v>14:74</x:v>
       </x:c>
       <x:c r="N26" s="4" t="str">
-        <x:v>77:78</x:v>
+        <x:v>77:77</x:v>
       </x:c>
       <x:c r="O26" s="4" t="str">
         <x:v>percentage</x:v>
@@ -2852,7 +2852,7 @@
         <x:v>Quantum</x:v>
       </x:c>
       <x:c r="F27" s="4" t="str">
-        <x:v>A79:AB610</x:v>
+        <x:v>A80:AB609</x:v>
       </x:c>
       <x:c r="G27" s="4" t="str">
         <x:v>S1b</x:v>
@@ -2864,7 +2864,7 @@
         <x:v>S1b.请问您目前长期居住在哪个城市？（单选）</x:v>
       </x:c>
       <x:c r="J27" s="4" t="str">
-        <x:v>79:80</x:v>
+        <x:v>80:81</x:v>
       </x:c>
       <x:c r="K27" s="4" t="str">
         <x:v>88,89</x:v>
@@ -2876,7 +2876,7 @@
         <x:v>92:607</x:v>
       </x:c>
       <x:c r="N27" s="4" t="str">
-        <x:v>609:610</x:v>
+        <x:v>609:609</x:v>
       </x:c>
       <x:c r="O27" s="4" t="str">
         <x:v>percentage</x:v>
@@ -2932,7 +2932,7 @@
         <x:v>Quantum</x:v>
       </x:c>
       <x:c r="F28" s="4" t="str">
-        <x:v>A611:AB638</x:v>
+        <x:v>A612:AB637</x:v>
       </x:c>
       <x:c r="G28" s="4" t="str">
         <x:v>Tier</x:v>
@@ -2944,7 +2944,7 @@
         <x:v>Tier.Tier</x:v>
       </x:c>
       <x:c r="J28" s="4" t="str">
-        <x:v>611:612</x:v>
+        <x:v>612:613</x:v>
       </x:c>
       <x:c r="K28" s="4" t="str">
         <x:v>620,621</x:v>
@@ -2956,7 +2956,7 @@
         <x:v>624:635</x:v>
       </x:c>
       <x:c r="N28" s="4" t="str">
-        <x:v>637:638</x:v>
+        <x:v>637:637</x:v>
       </x:c>
       <x:c r="O28" s="4" t="str">
         <x:v>percentage</x:v>

</xml_diff>